<commit_message>
I read the book till 100 Page. Topic Fibre Channel
</commit_message>
<xml_diff>
--- a/pral_cdh_hw_for_costing_v1.3for-Redhat.xlsx
+++ b/pral_cdh_hw_for_costing_v1.3for-Redhat.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tayyabr\Desktop\Presales-Working-August-2026-Onwards\PRAL\PRAL-RFP-September-26\Hardware Sizing\Server\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\system-engineering-portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7881C45D-8DA1-46B1-9467-8D96E684637E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
   </bookViews>
   <sheets>
     <sheet name="Virutal HW" sheetId="3" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Virutal HW'!$B$4:$F$35</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -326,7 +325,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -890,6 +889,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -937,9 +939,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -978,7 +977,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{089840E2-C711-407E-83CD-FAE9C60689B6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{089840E2-C711-407E-83CD-FAE9C60689B6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1296,90 +1295,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91421EC9-2BE0-45BB-BA7C-541601DD8189}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
   <dimension ref="A1:W57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.44140625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="38.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="6.109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.140625" style="2" customWidth="1"/>
     <col min="10" max="10" width="11" style="2" customWidth="1"/>
-    <col min="11" max="11" width="8.33203125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.6640625" style="2" customWidth="1"/>
-    <col min="14" max="14" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.44140625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="8.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.109375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="6.44140625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="5.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.88671875" style="2" customWidth="1"/>
-    <col min="21" max="21" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="26.88671875" customWidth="1"/>
+    <col min="11" max="11" width="8.28515625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.7109375" style="2" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.42578125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="8.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="6.42578125" style="2" customWidth="1"/>
+    <col min="19" max="19" width="5.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.85546875" style="2" customWidth="1"/>
+    <col min="21" max="21" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="26.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="J2" s="57" t="s">
+      <c r="J2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="59"/>
-      <c r="Q2" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
-      <c r="T2" s="61"/>
-      <c r="U2" s="62"/>
-    </row>
-    <row r="3" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G3" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" s="64"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="66" t="s">
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="60"/>
+      <c r="Q2" s="61" t="s">
+        <v>1</v>
+      </c>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="63"/>
+    </row>
+    <row r="3" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="64" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="65"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="67" t="s">
         <v>86</v>
       </c>
-      <c r="K3" s="68" t="s">
+      <c r="K3" s="69" t="s">
         <v>87</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M3" s="60" t="s">
+      <c r="M3" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="62"/>
-      <c r="Q3" s="70" t="s">
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="R3" s="71"/>
-      <c r="S3" s="70" t="s">
+      <c r="R3" s="72"/>
+      <c r="S3" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="T3" s="72"/>
-      <c r="U3" s="71"/>
-    </row>
-    <row r="4" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="T3" s="73"/>
+      <c r="U3" s="72"/>
+    </row>
+    <row r="4" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1404,8 +1403,8 @@
       <c r="I4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="67"/>
-      <c r="K4" s="69"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="70"/>
       <c r="L4" s="14" t="s">
         <v>15</v>
       </c>
@@ -1440,7 +1439,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B5" s="28" t="s">
         <v>23</v>
       </c>
@@ -1505,7 +1504,7 @@
       </c>
       <c r="U5" s="44"/>
     </row>
-    <row r="6" spans="2:23" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:23" ht="75" x14ac:dyDescent="0.25">
       <c r="B6" s="28" t="s">
         <v>23</v>
       </c>
@@ -1569,11 +1568,11 @@
         <v>10752</v>
       </c>
       <c r="U6" s="44"/>
-      <c r="V6" s="73" t="s">
+      <c r="V6" s="57" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B7" s="28" t="s">
         <v>23</v>
       </c>
@@ -1638,7 +1637,7 @@
       </c>
       <c r="U7" s="44"/>
     </row>
-    <row r="8" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="28" t="s">
         <v>23</v>
       </c>
@@ -1703,7 +1702,7 @@
       </c>
       <c r="U8" s="44"/>
     </row>
-    <row r="9" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="45"/>
       <c r="C9" s="46" t="s">
         <v>73</v>
@@ -1746,7 +1745,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B10" s="28"/>
       <c r="C10" s="51"/>
       <c r="D10" s="51"/>
@@ -1764,7 +1763,7 @@
       <c r="T10" s="27"/>
       <c r="U10" s="27"/>
     </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B11" s="28" t="s">
         <v>33</v>
       </c>
@@ -1829,7 +1828,7 @@
       </c>
       <c r="U11" s="44"/>
     </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B12" s="28" t="s">
         <v>33</v>
       </c>
@@ -1894,7 +1893,7 @@
       </c>
       <c r="U12" s="44"/>
     </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B13" s="28" t="s">
         <v>33</v>
       </c>
@@ -1960,7 +1959,7 @@
       <c r="U13" s="44"/>
       <c r="W13" s="30"/>
     </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B14" s="28" t="s">
         <v>33</v>
       </c>
@@ -2026,7 +2025,7 @@
       <c r="U14" s="44"/>
       <c r="W14" s="31"/>
     </row>
-    <row r="15" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B15" s="28" t="s">
         <v>33</v>
       </c>
@@ -2091,7 +2090,7 @@
       </c>
       <c r="U15" s="44"/>
     </row>
-    <row r="16" spans="2:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:23" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="32" t="s">
         <v>44</v>
       </c>
@@ -2156,7 +2155,7 @@
       </c>
       <c r="U16" s="44"/>
     </row>
-    <row r="17" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B17" s="32" t="s">
         <v>47</v>
       </c>
@@ -2221,7 +2220,7 @@
       </c>
       <c r="U17" s="44"/>
     </row>
-    <row r="18" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="32" t="s">
         <v>51</v>
       </c>
@@ -2283,7 +2282,7 @@
       </c>
       <c r="U18" s="44"/>
     </row>
-    <row r="19" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="45"/>
       <c r="C19" s="46" t="s">
         <v>73</v>
@@ -2327,7 +2326,7 @@
       </c>
       <c r="V19" s="55"/>
     </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B20" s="18" t="s">
         <v>19</v>
       </c>
@@ -2388,7 +2387,7 @@
       </c>
       <c r="U20" s="44"/>
     </row>
-    <row r="21" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B21" s="32" t="s">
         <v>51</v>
       </c>
@@ -2451,7 +2450,7 @@
       </c>
       <c r="U21" s="44"/>
     </row>
-    <row r="22" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="32" t="s">
         <v>51</v>
       </c>
@@ -2513,7 +2512,7 @@
       </c>
       <c r="U22" s="44"/>
     </row>
-    <row r="23" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B23" s="56" t="s">
         <v>51</v>
       </c>
@@ -2550,7 +2549,7 @@
       <c r="T23" s="27"/>
       <c r="U23" s="44"/>
     </row>
-    <row r="24" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B24" s="56" t="s">
         <v>51</v>
       </c>
@@ -2587,7 +2586,7 @@
       <c r="T24" s="27"/>
       <c r="U24" s="44"/>
     </row>
-    <row r="25" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B25" s="32" t="s">
         <v>51</v>
       </c>
@@ -2637,7 +2636,7 @@
       <c r="T25" s="27"/>
       <c r="U25" s="44"/>
     </row>
-    <row r="26" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B26" s="32"/>
       <c r="E26" s="4" t="s">
         <v>67</v>
@@ -2657,7 +2656,7 @@
       <c r="S26" s="27"/>
       <c r="U26" s="44"/>
     </row>
-    <row r="27" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="32"/>
       <c r="E27" s="4" t="s">
         <v>84</v>
@@ -2677,7 +2676,7 @@
       <c r="S27" s="27"/>
       <c r="U27" s="44"/>
     </row>
-    <row r="28" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="45"/>
       <c r="C28" s="46" t="s">
         <v>73</v>
@@ -2721,7 +2720,7 @@
       </c>
       <c r="V28" s="55"/>
     </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="52"/>
       <c r="E29" s="4"/>
       <c r="G29" s="27"/>
@@ -2738,7 +2737,7 @@
       <c r="T29" s="23"/>
       <c r="U29" s="44"/>
     </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" s="28" t="s">
         <v>19</v>
       </c>
@@ -2800,7 +2799,7 @@
       </c>
       <c r="U30" s="44"/>
     </row>
-    <row r="31" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" s="28" t="s">
         <v>23</v>
       </c>
@@ -2865,7 +2864,7 @@
       </c>
       <c r="U31" s="44"/>
     </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" s="28" t="s">
         <v>23</v>
       </c>
@@ -2930,7 +2929,7 @@
       </c>
       <c r="U32" s="44"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B33" s="28" t="s">
         <v>33</v>
       </c>
@@ -2995,7 +2994,7 @@
       </c>
       <c r="U33" s="44"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B34" s="32" t="s">
         <v>44</v>
       </c>
@@ -3060,7 +3059,7 @@
       </c>
       <c r="U34" s="44"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B35" s="32" t="s">
         <v>47</v>
       </c>
@@ -3125,7 +3124,7 @@
       </c>
       <c r="U35" s="44"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B36" s="32" t="s">
         <v>51</v>
       </c>
@@ -3187,7 +3186,7 @@
       </c>
       <c r="U36" s="44"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B37" s="32" t="s">
         <v>51</v>
       </c>
@@ -3249,7 +3248,7 @@
       </c>
       <c r="U37" s="44"/>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B38" s="32" t="s">
         <v>51</v>
       </c>
@@ -3311,7 +3310,7 @@
       </c>
       <c r="U38" s="44"/>
     </row>
-    <row r="39" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="32" t="s">
         <v>51</v>
       </c>
@@ -3360,7 +3359,7 @@
       <c r="T39" s="26"/>
       <c r="U39" s="44"/>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B40" s="45"/>
       <c r="C40" s="46" t="s">
         <v>73</v>
@@ -3404,7 +3403,7 @@
       </c>
       <c r="V40" s="55"/>
     </row>
-    <row r="41" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="28"/>
       <c r="G41" s="27"/>
       <c r="H41" s="26"/>
@@ -3420,7 +3419,7 @@
       <c r="T41" s="36"/>
       <c r="U41" s="44"/>
     </row>
-    <row r="42" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="38" t="s">
         <v>69</v>
       </c>
@@ -3444,26 +3443,26 @@
       <c r="T42" s="42"/>
       <c r="U42" s="53"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="E43"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B44" s="2"/>
       <c r="E44"/>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
       <c r="E45"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B46" s="2"/>
     </row>
-    <row r="47" spans="1:22" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E47" s="4"/>
       <c r="G47" s="54"/>
       <c r="H47" s="54"/>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -3471,49 +3470,49 @@
       <c r="F48" s="4"/>
       <c r="G48" s="54"/>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
     </row>
-    <row r="51" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="F51" s="3"/>
       <c r="U51"/>
       <c r="V51"/>
       <c r="W51"/>
     </row>
-    <row r="52" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="U52"/>
       <c r="V52"/>
       <c r="W52"/>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
     </row>
-    <row r="54" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="F54" s="3"/>
       <c r="U54"/>
       <c r="V54"/>
       <c r="W54"/>
     </row>
-    <row r="55" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="F55" s="3"/>
       <c r="U55"/>
       <c r="V55"/>
       <c r="W55"/>
     </row>
-    <row r="56" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -3525,7 +3524,7 @@
       <c r="V56"/>
       <c r="W56"/>
     </row>
-    <row r="57" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>

</xml_diff>